<commit_message>
Rename defect-table human columns to human_reviewer_verdict and human_reviewer_note.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/paper_experiments/data/defects_table.xlsx
+++ b/paper_experiments/data/defects_table.xlsx
@@ -496,12 +496,12 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>your_verdict</t>
+          <t>human_reviewer_verdict</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>your_note</t>
+          <t>human_reviewer_note</t>
         </is>
       </c>
     </row>

</xml_diff>